<commit_message>
Re-link project after folder restructuring
</commit_message>
<xml_diff>
--- a/CPI.xlsx
+++ b/CPI.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29819"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://barnard0-my.sharepoint.com/personal/ksemm_barnard_edu/Documents/Manuscripts/Utility Burden/"/>
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,6 +37,18 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Annual Average CPI</t>
+  </si>
+  <si>
+    <t>Percentage Change</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
   <si>
     <t> 2013</t>
   </si>
@@ -73,24 +85,12 @@
   <si>
     <t> 2024</t>
   </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Annual Average CPI</t>
-  </si>
-  <si>
-    <t>Percentage Change</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -472,25 +472,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A099947-736F-834D-A855-B65A0A5D4421}">
   <dimension ref="A1:C113"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <cols>
-    <col min="1" max="1" width="11.1640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.1640625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="11.125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.125" style="3" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3">
       <c r="A1" s="5" t="s">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="20.100000000000001">
       <c r="A2" s="6">
         <v>1913</v>
       </c>
@@ -498,10 +498,10 @@
         <v>9.9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="20.100000000000001">
       <c r="A3" s="6">
         <v>1914</v>
       </c>
@@ -512,7 +512,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="20.100000000000001">
       <c r="A4" s="6">
         <v>1915</v>
       </c>
@@ -523,7 +523,7 @@
         <v>8.9999999999999993E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="20.100000000000001">
       <c r="A5" s="6">
         <v>1916</v>
       </c>
@@ -534,7 +534,7 @@
         <v>7.6999999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="20.100000000000001">
       <c r="A6" s="6">
         <v>1917</v>
       </c>
@@ -545,7 +545,7 @@
         <v>0.17799999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="20.100000000000001">
       <c r="A7" s="6">
         <v>1918</v>
       </c>
@@ -556,7 +556,7 @@
         <v>0.17299999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="20.100000000000001">
       <c r="A8" s="6">
         <v>1919</v>
       </c>
@@ -567,7 +567,7 @@
         <v>0.152</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="20.100000000000001">
       <c r="A9" s="6">
         <v>1920</v>
       </c>
@@ -578,7 +578,7 @@
         <v>0.156</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="20.100000000000001">
       <c r="A10" s="6">
         <v>1921</v>
       </c>
@@ -589,7 +589,7 @@
         <v>-0.109</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="20.100000000000001">
       <c r="A11" s="6">
         <v>1922</v>
       </c>
@@ -600,7 +600,7 @@
         <v>-6.2E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="20.100000000000001">
       <c r="A12" s="6">
         <v>1923</v>
       </c>
@@ -611,7 +611,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" ht="20.100000000000001">
       <c r="A13" s="6">
         <v>1924</v>
       </c>
@@ -622,7 +622,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" ht="20.100000000000001">
       <c r="A14" s="6">
         <v>1925</v>
       </c>
@@ -633,7 +633,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" ht="20.100000000000001">
       <c r="A15" s="6">
         <v>1926</v>
       </c>
@@ -644,7 +644,7 @@
         <v>8.9999999999999993E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" ht="20.100000000000001">
       <c r="A16" s="6">
         <v>1927</v>
       </c>
@@ -655,7 +655,7 @@
         <v>-1.9E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" ht="20.100000000000001">
       <c r="A17" s="6">
         <v>1928</v>
       </c>
@@ -666,7 +666,7 @@
         <v>-1.2E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" ht="20.100000000000001">
       <c r="A18" s="6">
         <v>1929</v>
       </c>
@@ -677,7 +677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" ht="20.100000000000001">
       <c r="A19" s="6">
         <v>1930</v>
       </c>
@@ -688,7 +688,7 @@
         <v>-2.7E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" ht="20.100000000000001">
       <c r="A20" s="6">
         <v>1931</v>
       </c>
@@ -699,7 +699,7 @@
         <v>-8.8999999999999996E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" ht="20.100000000000001">
       <c r="A21" s="6">
         <v>1932</v>
       </c>
@@ -710,7 +710,7 @@
         <v>-0.10299999999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" ht="20.100000000000001">
       <c r="A22" s="6">
         <v>1933</v>
       </c>
@@ -721,7 +721,7 @@
         <v>-5.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" ht="20.100000000000001">
       <c r="A23" s="6">
         <v>1934</v>
       </c>
@@ -732,7 +732,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" ht="20.100000000000001">
       <c r="A24" s="6">
         <v>1935</v>
       </c>
@@ -743,7 +743,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" ht="20.100000000000001">
       <c r="A25" s="6">
         <v>1936</v>
       </c>
@@ -754,7 +754,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" ht="20.100000000000001">
       <c r="A26" s="6">
         <v>1937</v>
       </c>
@@ -765,7 +765,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" ht="20.100000000000001">
       <c r="A27" s="6">
         <v>1938</v>
       </c>
@@ -776,7 +776,7 @@
         <v>-0.02</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" ht="20.100000000000001">
       <c r="A28" s="6">
         <v>1939</v>
       </c>
@@ -787,7 +787,7 @@
         <v>-1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" ht="20.100000000000001">
       <c r="A29" s="6">
         <v>1940</v>
       </c>
@@ -798,7 +798,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" ht="20.100000000000001">
       <c r="A30" s="6">
         <v>1941</v>
       </c>
@@ -809,7 +809,7 @@
         <v>5.0999999999999997E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" ht="20.100000000000001">
       <c r="A31" s="6">
         <v>1942</v>
       </c>
@@ -820,7 +820,7 @@
         <v>0.109</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" ht="20.100000000000001">
       <c r="A32" s="6">
         <v>1943</v>
       </c>
@@ -831,7 +831,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" ht="20.100000000000001">
       <c r="A33" s="6">
         <v>1944</v>
       </c>
@@ -842,7 +842,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" ht="20.100000000000001">
       <c r="A34" s="6">
         <v>1945</v>
       </c>
@@ -853,7 +853,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" ht="20.100000000000001">
       <c r="A35" s="6">
         <v>1946</v>
       </c>
@@ -864,7 +864,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" ht="20.100000000000001">
       <c r="A36" s="6">
         <v>1947</v>
       </c>
@@ -875,7 +875,7 @@
         <v>0.14399999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" ht="20.100000000000001">
       <c r="A37" s="6">
         <v>1948</v>
       </c>
@@ -886,7 +886,7 @@
         <v>7.6999999999999999E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3" ht="20.100000000000001">
       <c r="A38" s="6">
         <v>1949</v>
       </c>
@@ -897,7 +897,7 @@
         <v>-0.01</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" ht="20.100000000000001">
       <c r="A39" s="6">
         <v>1950</v>
       </c>
@@ -908,7 +908,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3" ht="20.100000000000001">
       <c r="A40" s="6">
         <v>1951</v>
       </c>
@@ -919,7 +919,7 @@
         <v>7.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:3" ht="20.100000000000001">
       <c r="A41" s="6">
         <v>1952</v>
       </c>
@@ -930,7 +930,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" ht="20.100000000000001">
       <c r="A42" s="6">
         <v>1953</v>
       </c>
@@ -941,7 +941,7 @@
         <v>8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" ht="20.100000000000001">
       <c r="A43" s="6">
         <v>1954</v>
       </c>
@@ -952,7 +952,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" ht="20.100000000000001">
       <c r="A44" s="6">
         <v>1955</v>
       </c>
@@ -963,7 +963,7 @@
         <v>-3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3" ht="20.100000000000001">
       <c r="A45" s="6">
         <v>1956</v>
       </c>
@@ -974,7 +974,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" ht="20.100000000000001">
       <c r="A46" s="6">
         <v>1957</v>
       </c>
@@ -985,7 +985,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:3" ht="20.100000000000001">
       <c r="A47" s="6">
         <v>1958</v>
       </c>
@@ -996,7 +996,7 @@
         <v>2.7E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:3" ht="20.100000000000001">
       <c r="A48" s="6">
         <v>1959</v>
       </c>
@@ -1007,7 +1007,7 @@
         <v>1.0800000000000001E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:3" ht="20.100000000000001">
       <c r="A49" s="6">
         <v>1960</v>
       </c>
@@ -1018,7 +1018,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3" ht="20.100000000000001">
       <c r="A50" s="6">
         <v>1961</v>
       </c>
@@ -1029,7 +1029,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:3" ht="20.100000000000001">
       <c r="A51" s="6">
         <v>1962</v>
       </c>
@@ -1040,7 +1040,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:3" ht="20.100000000000001">
       <c r="A52" s="6">
         <v>1963</v>
       </c>
@@ -1051,7 +1051,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:3" ht="20.100000000000001">
       <c r="A53" s="6">
         <v>1964</v>
       </c>
@@ -1062,7 +1062,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:3" ht="20.100000000000001">
       <c r="A54" s="6">
         <v>1965</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:3" ht="20.100000000000001">
       <c r="A55" s="6">
         <v>1966</v>
       </c>
@@ -1084,7 +1084,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:3" ht="20.100000000000001">
       <c r="A56" s="6">
         <v>1967</v>
       </c>
@@ -1095,7 +1095,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:3" ht="20.100000000000001">
       <c r="A57" s="6">
         <v>1968</v>
       </c>
@@ -1106,7 +1106,7 @@
         <v>4.2999999999999997E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:3" ht="20.100000000000001">
       <c r="A58" s="6">
         <v>1969</v>
       </c>
@@ -1117,7 +1117,7 @@
         <v>5.5E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:3" ht="20.100000000000001">
       <c r="A59" s="6">
         <v>1970</v>
       </c>
@@ -1128,7 +1128,7 @@
         <v>5.8000000000000003E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:3" ht="20.100000000000001">
       <c r="A60" s="6">
         <v>1971</v>
       </c>
@@ -1139,7 +1139,7 @@
         <v>4.2999999999999997E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:3" ht="20.100000000000001">
       <c r="A61" s="6">
         <v>1972</v>
       </c>
@@ -1150,7 +1150,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:3" ht="20.100000000000001">
       <c r="A62" s="6">
         <v>1973</v>
       </c>
@@ -1161,7 +1161,7 @@
         <v>6.2E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:3" ht="20.100000000000001">
       <c r="A63" s="6">
         <v>1974</v>
       </c>
@@ -1172,7 +1172,7 @@
         <v>0.111</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:3" ht="20.100000000000001">
       <c r="A64" s="6">
         <v>1975</v>
       </c>
@@ -1183,7 +1183,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:3" ht="20.100000000000001">
       <c r="A65" s="6">
         <v>1976</v>
       </c>
@@ -1194,7 +1194,7 @@
         <v>5.7000000000000002E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:3" ht="20.100000000000001">
       <c r="A66" s="6">
         <v>1977</v>
       </c>
@@ -1205,7 +1205,7 @@
         <v>6.5000000000000002E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:3" ht="20.100000000000001">
       <c r="A67" s="6">
         <v>1978</v>
       </c>
@@ -1216,7 +1216,7 @@
         <v>7.5999999999999998E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:3" ht="20.100000000000001">
       <c r="A68" s="6">
         <v>1979</v>
       </c>
@@ -1227,7 +1227,7 @@
         <v>0.113</v>
       </c>
     </row>
-    <row r="69" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:3" ht="20.100000000000001">
       <c r="A69" s="6">
         <v>1980</v>
       </c>
@@ -1238,7 +1238,7 @@
         <v>0.13500000000000001</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:3" ht="20.100000000000001">
       <c r="A70" s="6">
         <v>1981</v>
       </c>
@@ -1249,7 +1249,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:3" ht="20.100000000000001">
       <c r="A71" s="6">
         <v>1982</v>
       </c>
@@ -1260,7 +1260,7 @@
         <v>6.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:3" ht="20.100000000000001">
       <c r="A72" s="6">
         <v>1983</v>
       </c>
@@ -1271,7 +1271,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:3" ht="20.100000000000001">
       <c r="A73" s="6">
         <v>1984</v>
       </c>
@@ -1282,7 +1282,7 @@
         <v>4.2999999999999997E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:3" ht="20.100000000000001">
       <c r="A74" s="6">
         <v>1985</v>
       </c>
@@ -1293,7 +1293,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:3" ht="20.100000000000001">
       <c r="A75" s="6">
         <v>1986</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:3" ht="20.100000000000001">
       <c r="A76" s="6">
         <v>1987</v>
       </c>
@@ -1315,7 +1315,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:3" ht="20.100000000000001">
       <c r="A77" s="6">
         <v>1988</v>
       </c>
@@ -1326,7 +1326,7 @@
         <v>4.1000000000000002E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:3" ht="20.100000000000001">
       <c r="A78" s="6">
         <v>1989</v>
       </c>
@@ -1337,7 +1337,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:3" ht="20.100000000000001">
       <c r="A79" s="6">
         <v>1990</v>
       </c>
@@ -1348,7 +1348,7 @@
         <v>5.3999999999999999E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:3" ht="20.100000000000001">
       <c r="A80" s="6">
         <v>1991</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>4.2000000000000003E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:3" ht="20.100000000000001">
       <c r="A81" s="6">
         <v>1992</v>
       </c>
@@ -1370,7 +1370,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:3" ht="20.100000000000001">
       <c r="A82" s="6">
         <v>1993</v>
       </c>
@@ -1381,7 +1381,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:3" ht="20.100000000000001">
       <c r="A83" s="6">
         <v>1994</v>
       </c>
@@ -1392,7 +1392,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:3" ht="20.100000000000001">
       <c r="A84" s="6">
         <v>1995</v>
       </c>
@@ -1403,7 +1403,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:3" ht="20.100000000000001">
       <c r="A85" s="6">
         <v>1996</v>
       </c>
@@ -1414,7 +1414,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:3" ht="20.100000000000001">
       <c r="A86" s="6">
         <v>1997</v>
       </c>
@@ -1425,7 +1425,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:3" ht="20.100000000000001">
       <c r="A87" s="6">
         <v>1998</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:3" ht="20.100000000000001">
       <c r="A88" s="6">
         <v>1999</v>
       </c>
@@ -1447,7 +1447,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:3" ht="20.100000000000001">
       <c r="A89" s="6">
         <v>2000</v>
       </c>
@@ -1458,7 +1458,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:3" ht="20.100000000000001">
       <c r="A90" s="6">
         <v>2001</v>
       </c>
@@ -1469,7 +1469,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:3" ht="20.100000000000001">
       <c r="A91" s="6">
         <v>2002</v>
       </c>
@@ -1480,7 +1480,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:3" ht="20.100000000000001">
       <c r="A92" s="6">
         <v>2003</v>
       </c>
@@ -1491,7 +1491,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:3" ht="20.100000000000001">
       <c r="A93" s="6">
         <v>2004</v>
       </c>
@@ -1502,7 +1502,7 @@
         <v>2.7E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:3" ht="20.100000000000001">
       <c r="A94" s="6">
         <v>2005</v>
       </c>
@@ -1513,7 +1513,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:3" ht="20.100000000000001">
       <c r="A95" s="6">
         <v>2006</v>
       </c>
@@ -1524,7 +1524,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:3" ht="20.100000000000001">
       <c r="A96" s="6">
         <v>2007</v>
       </c>
@@ -1535,7 +1535,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:3" ht="20.100000000000001">
       <c r="A97" s="6">
         <v>2008</v>
       </c>
@@ -1546,7 +1546,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:3" ht="20.100000000000001">
       <c r="A98" s="6">
         <v>2009</v>
       </c>
@@ -1557,7 +1557,7 @@
         <v>-4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="99" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:3" ht="20.100000000000001">
       <c r="A99" s="6">
         <v>2010</v>
       </c>
@@ -1568,7 +1568,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="100" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:3" ht="20.100000000000001">
       <c r="A100" s="6">
         <v>2011</v>
       </c>
@@ -1579,7 +1579,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="101" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:3" ht="20.100000000000001">
       <c r="A101" s="6">
         <v>2012</v>
       </c>
@@ -1590,9 +1590,9 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="102" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:3" ht="20.100000000000001">
       <c r="A102" s="6" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B102" s="4">
         <v>233</v>
@@ -1601,9 +1601,9 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="103" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:3" ht="20.100000000000001">
       <c r="A103" s="6" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B103" s="4">
         <v>236.7</v>
@@ -1612,9 +1612,9 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:3" ht="20.100000000000001">
       <c r="A104" s="6" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B104" s="4">
         <v>237</v>
@@ -1623,9 +1623,9 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:3" ht="20.100000000000001">
       <c r="A105" s="6" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B105" s="4">
         <v>240</v>
@@ -1634,9 +1634,9 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="106" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:3" ht="20.100000000000001">
       <c r="A106" s="6" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B106" s="4">
         <v>245.1</v>
@@ -1645,9 +1645,9 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="107" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:3" ht="20.100000000000001">
       <c r="A107" s="6" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B107" s="4">
         <v>251.1</v>
@@ -1656,9 +1656,9 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="108" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:3" ht="20.100000000000001">
       <c r="A108" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B108" s="4">
         <v>255.7</v>
@@ -1667,9 +1667,9 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:3" ht="20.100000000000001">
       <c r="A109" s="6" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B109" s="4">
         <v>258.8</v>
@@ -1678,9 +1678,9 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="110" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:3" ht="20.100000000000001">
       <c r="A110" s="6" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B110" s="4">
         <v>271</v>
@@ -1689,9 +1689,9 @@
         <v>4.7E-2</v>
       </c>
     </row>
-    <row r="111" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:3" ht="20.100000000000001">
       <c r="A111" s="6" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B111" s="4">
         <v>292.7</v>
@@ -1700,9 +1700,9 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="112" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:3" ht="20.100000000000001">
       <c r="A112" s="6" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B112" s="4">
         <v>304.7</v>
@@ -1711,9 +1711,9 @@
         <v>4.1000000000000002E-2</v>
       </c>
     </row>
-    <row r="113" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:3" ht="20.100000000000001">
       <c r="A113" s="6" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B113" s="4">
         <v>314.39999999999998</v>

</xml_diff>